<commit_message>
chore(samples): update parameter_ref_sample to kebab-case names and FGR-* feature codes
- Column order: Parameter Name first, Feature Name last
- Parameter names: kebab-case (e.g. carrier-aggregation-enable)
- Feature names: FGR-XX0000 format (e.g. FGR-HO0101, FGR-RS0101)
- 11 rows: HO×3, CA×3, RACH×2, BWP×2, TTT×1
- Update tests to match new sample data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/spar/data/samples/parameter_ref_sample.xlsx
+++ b/spar/data/samples/parameter_ref_sample.xlsx
@@ -425,65 +425,65 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Parameter Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>YANG Path</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Feature Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>YANG Path</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Parameter Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Min</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HO</t>
+          <t>handover-preparation-timer</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -493,33 +493,33 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>hoPrepTimerHO</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
           <t>INTEGER</t>
         </is>
       </c>
+      <c r="D2" t="n">
+        <v>100</v>
+      </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
         <v>1023</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Handover preparation timer value in ms. Triggered when UE measurement report received.</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Handover preparation timer value in ms. Triggered when UE measurement report received.</t>
+          <t>FGR-HO0101</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HO</t>
+          <t>handover-a3-offset</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,33 +529,33 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>hoA3Offset</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
           <t>INTEGER</t>
         </is>
       </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>-30</v>
       </c>
       <c r="F3" t="n">
-        <v>-30</v>
-      </c>
-      <c r="G3" t="n">
         <v>30</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>A3 event offset for intra-frequency handover trigger (unit: 0.5 dB).</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>A3 event offset for intra-frequency handover trigger (unit: 0.5 dB).</t>
+          <t>FGR-HO0101</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HO</t>
+          <t>handover-hysteresis</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -565,33 +565,33 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>hoHysteresis</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
           <t>INTEGER</t>
         </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
         <v>30</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Hysteresis value for A3 event evaluation (unit: 0.5 dB).</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Hysteresis value for A3 event evaluation (unit: 0.5 dB).</t>
+          <t>FGR-HO0101</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>carrier-aggregation-enable</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -601,33 +601,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>maxNumScell</t>
+          <t>BOOLEAN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>7</v>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Enables carrier aggregation for the cell. Requires compatible UE capability.</t>
+        </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Maximum number of secondary cells allowed per UE in CA.</t>
+          <t>FGR-CA0201</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>carrier-aggregation-max-scell</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -637,69 +633,69 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>scellActivationTimer</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
           <t>INTEGER</t>
         </is>
       </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
       <c r="E6" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2000</v>
+        <v>7</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Maximum number of secondary cells allowed per UE in CA.</t>
+        </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SCell activation timer value in ms after CA configuration.</t>
+          <t>FGR-CA0201</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RACH</t>
+          <t>scell-activation-timer</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ManagedElement/GNBDUFunction/NRCellDU/RachConfig</t>
+          <t>ManagedElement/GNBCUCPFunction/NRCellCU/CarrierAggConfig</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>preambleInitialReceivedTargetPower</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
           <t>INTEGER</t>
         </is>
       </c>
+      <c r="D7" t="n">
+        <v>200</v>
+      </c>
       <c r="E7" t="n">
-        <v>-104</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>-202</v>
-      </c>
-      <c r="G7" t="n">
-        <v>-60</v>
+        <v>2000</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>SCell activation timer value in ms after CA configuration.</t>
+        </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Initial target received power for preamble in dBm.</t>
+          <t>FGR-CA0201</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RACH</t>
+          <t>rach-preamble-target-power</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -709,65 +705,65 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>powerRampingStep</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>ENUMERATION</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2dB</t>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>-104</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-202</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-60</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Initial target received power for preamble in dBm.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Power ramping step for preamble retransmission. Values: 0dB, 2dB, 4dB, 6dB.</t>
+          <t>FGR-RS0101</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BWP</t>
+          <t>rach-power-ramping-step</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ManagedElement/GNBDUFunction/NRCellDU/BWPConfig</t>
+          <t>ManagedElement/GNBDUFunction/NRCellDU/RachConfig</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>bwpInactivityTimer</t>
+          <t>ENUMERATION</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>2560</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>2560</v>
+          <t>2dB</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Power ramping step for preamble retransmission. Values: 0dB, 2dB, 4dB, 6dB.</t>
+        </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Inactivity timer for returning to default BWP (ms). 0 disables the timer.</t>
+          <t>FGR-RS0101</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BWP</t>
+          <t>bwp-inactivity-timer</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -777,58 +773,94 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>initialBWPDLBandwidth</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
           <t>INTEGER</t>
         </is>
       </c>
+      <c r="D10" t="n">
+        <v>2560</v>
+      </c>
       <c r="E10" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="n">
-        <v>275</v>
+        <v>2560</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Inactivity timer for returning to default BWP (ms). 0 disables the timer.</t>
+        </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Initial downlink BWP bandwidth in resource blocks.</t>
+          <t>FGR-BW0301</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TTT</t>
+          <t>bwp-initial-dl-bandwidth</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBDUFunction/NRCellDU/BWPConfig</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>275</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Initial downlink BWP bandwidth in resource blocks.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>FGR-BW0301</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>meas-time-to-trigger</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>ManagedElement/GNBCUCPFunction/NRCellCU/MeasConfig</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>timeToTrigger</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>ENUMERATION</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>100ms</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Time-to-trigger for event evaluation. Values: 0ms, 40ms, 64ms, 80ms, 100ms, 128ms, 160ms, 256ms, 320ms, 480ms, 512ms, 640ms.</t>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Time-to-trigger for event evaluation. Values: 0ms 40ms 64ms 80ms 100ms 128ms 160ms 256ms 320ms 480ms 512ms 640ms.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>FGR-HO0102</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(parser): expand parameter Excel schema to 20-column format
Real parameter reference files use Hierarchy/Attribute Key/Range/etc.
instead of the old YANG Path/Parameter Name/Min/Max layout. Updates
aliases, ParameterRecord fields, chunk text, and sample fixture to match.
</commit_message>
<xml_diff>
--- a/spar/data/samples/parameter_ref_sample.xlsx
+++ b/spar/data/samples/parameter_ref_sample.xlsx
@@ -40,6 +40,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -425,442 +426,968 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Parameter Name</t>
+          <t>Hierarchy</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>YANG Path</t>
+          <t>Parameter Description</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Attribute Key</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Leaf Status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Min</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Feature Name</t>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Default Value</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Bandwidth-Dependancy</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Config value</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Restriction</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Service Impact</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Real time change</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Parameter-Family</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Related Feature ID</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>User Level</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBCUCPFunction/NRCellCU/HandoverConfig</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Handover preparation timer value in ms. Triggered when UE measurement report received.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>handover-preparation-timer</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBCUCPFunction/NRCellCU/HandoverConfig</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ms</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>100</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1023</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Handover preparation timer value in ms. Triggered when UE measurement report received.</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
+          <t>0..1023</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Handover</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
           <t>FGR-HO0101</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBCUCPFunction/NRCellCU/HandoverConfig</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A3 event offset for intra-frequency handover trigger (unit: 0.5 dB).</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>handover-a3-offset</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBCUCPFunction/NRCellCU/HandoverConfig</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.5 dB</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" t="n">
-        <v>-30</v>
-      </c>
-      <c r="F3" t="n">
-        <v>30</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>A3 event offset for intra-frequency handover trigger (unit: 0.5 dB).</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
+          <t>-30..30</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Handover</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
           <t>FGR-HO0101</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBCUCPFunction/NRCellCU/HandoverConfig</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Hysteresis value for A3 event evaluation (unit: 0.5 dB).</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>handover-hysteresis</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBCUCPFunction/NRCellCU/HandoverConfig</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.5 dB</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>30</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Hysteresis value for A3 event evaluation (unit: 0.5 dB).</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
+          <t>0..30</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Handover</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
           <t>FGR-HO0101</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBCUCPFunction/NRCellCU/CarrierAggConfig</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Enables carrier aggregation for the cell. Requires compatible UE capability.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>carrier-aggregation-enable</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBCUCPFunction/NRCellCU/CarrierAggConfig</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
         <is>
           <t>BOOLEAN</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Enables carrier aggregation for the cell. Requires compatible UE capability.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Carrier Aggregation</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
         <is>
           <t>FGR-CA0201</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBCUCPFunction/NRCellCU/CarrierAggConfig</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Maximum number of secondary cells allowed per UE in CA.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>carrier-aggregation-max-scell</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBCUCPFunction/NRCellCU/CarrierAggConfig</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>7</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Maximum number of secondary cells allowed per UE in CA.</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
+          <t>1..7</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Carrier Aggregation</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
           <t>FGR-CA0201</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBCUCPFunction/NRCellCU/CarrierAggConfig</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SCell activation timer value in ms after CA configuration.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>scell-activation-timer</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBCUCPFunction/NRCellCU/CarrierAggConfig</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ms</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>200</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>SCell activation timer value in ms after CA configuration.</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
+          <t>0..2000</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Carrier Aggregation</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
           <t>FGR-CA0201</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBDUFunction/NRCellDU/RachConfig</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Initial target received power for preamble in dBm.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>rach-preamble-target-power</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBDUFunction/NRCellDU/RachConfig</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>dBm</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>-104</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-202</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-60</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Initial target received power for preamble in dBm.</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
+          <t>-202..-60</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>-104</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Random Access</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
           <t>FGR-RS0101</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBDUFunction/NRCellDU/RachConfig</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Power ramping step for preamble retransmission. Values: 0dB, 2dB, 4dB, 6dB.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>rach-power-ramping-step</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBDUFunction/NRCellDU/RachConfig</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
         <is>
           <t>ENUMERATION</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0dB, 2dB, 4dB, 6dB</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
         <is>
           <t>2dB</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Power ramping step for preamble retransmission. Values: 0dB, 2dB, 4dB, 6dB.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Random Access</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
         <is>
           <t>FGR-RS0101</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBDUFunction/NRCellDU/BWPConfig</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Inactivity timer for returning to default BWP (ms). 0 disables the timer.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>bwp-inactivity-timer</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBDUFunction/NRCellDU/BWPConfig</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ms</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>2560</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>2560</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Inactivity timer for returning to default BWP (ms). 0 disables the timer.</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
+          <t>0..2560</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2560</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Bandwidth Part</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
           <t>FGR-BW0301</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBDUFunction/NRCellDU/BWPConfig</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Initial downlink BWP bandwidth in resource blocks.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>bwp-initial-dl-bandwidth</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBDUFunction/NRCellDU/BWPConfig</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>52</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="n">
-        <v>275</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Initial downlink BWP bandwidth in resource blocks.</t>
-        </is>
-      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
+          <t>1..275</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Bandwidth Part</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
           <t>FGR-BW0301</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>ManagedElement/GNBCUCPFunction/NRCellCU/MeasConfig</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Time-to-trigger for event evaluation. Values: 0ms 40ms 64ms 80ms 100ms 128ms 160ms 256ms 320ms 480ms 512ms 640ms.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>meas-time-to-trigger</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>ManagedElement/GNBCUCPFunction/NRCellCU/MeasConfig</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
         <is>
           <t>ENUMERATION</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0ms 40ms 64ms 80ms 100ms 128ms 160ms 256ms 320ms 480ms 512ms 640ms</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
         <is>
           <t>100ms</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Time-to-trigger for event evaluation. Values: 0ms 40ms 64ms 80ms 100ms 128ms 160ms 256ms 320ms 480ms 512ms 640ms.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Handover</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
         <is>
           <t>FGR-HO0102</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Expert</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(parser): correct parameter Excel schema to 22-column format
Parameter/Description and Attribute/Key Leaf/Status were incorrectly
merged in the previous schema. Splits them into distinct columns per
actual Samsung RAN spec layout.

- attribute: leaf / leaf-list
- key_leaf: X / O
- status: current / deprecated
</commit_message>
<xml_diff>
--- a/spar/data/samples/parameter_ref_sample.xlsx
+++ b/spar/data/samples/parameter_ref_sample.xlsx
@@ -426,29 +426,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T12"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="21" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,95 +461,105 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Parameter Description</t>
+          <t>Parameter</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Attribute Key</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Leaf Status</t>
+          <t>Attribute</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Key Leaf</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Pattern</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Default Value</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Bandwidth-Dependancy</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Config value</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Restriction</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Service Impact</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Real time change</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Parameter-Family</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Related Feature ID</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>User Level</t>
         </is>
@@ -561,71 +573,81 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>handover-preparation-timer</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Handover preparation timer value in ms. Triggered when UE measurement report received.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>handover-preparation-timer</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>leaf</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
         <is>
           <t>0..1023</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Handover</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>FGR-HO0101</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
@@ -639,71 +661,81 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>handover-a3-offset</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>A3 event offset for intra-frequency handover trigger (unit: 0.5 dB).</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>handover-a3-offset</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>leaf</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>0.5 dB</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
         <is>
           <t>-30..30</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>Handover</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>FGR-HO0101</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
@@ -717,71 +749,81 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>handover-hysteresis</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Hysteresis value for A3 event evaluation (unit: 0.5 dB).</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>handover-hysteresis</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>leaf</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>0.5 dB</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>0..30</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Handover</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>FGR-HO0101</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
@@ -795,63 +837,73 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>carrier-aggregation-enable</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Enables carrier aggregation for the cell. Requires compatible UE capability.</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>carrier-aggregation-enable</t>
-        </is>
-      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>RW</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>leaf</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>BOOLEAN</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>Carrier Aggregation</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>FGR-CA0201</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
@@ -865,67 +917,77 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>carrier-aggregation-max-scell</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>Maximum number of secondary cells allowed per UE in CA.</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>carrier-aggregation-max-scell</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>RW</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>leaf</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>INTEGER</t>
+          <t>current</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>1..7</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>Carrier Aggregation</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>FGR-CA0201</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
@@ -939,71 +1001,81 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>scell-activation-timer</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>SCell activation timer value in ms after CA configuration.</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>scell-activation-timer</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>leaf</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
         <is>
           <t>0..2000</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>Carrier Aggregation</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>FGR-CA0201</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
@@ -1017,71 +1089,81 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>rach-preamble-target-power</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Initial target received power for preamble in dBm.</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>rach-preamble-target-power</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>leaf</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
           <t>dBm</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
         <is>
           <t>-202..-60</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>-104</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>Random Access</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>FGR-RS0101</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
@@ -1095,67 +1177,77 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Power ramping step for preamble retransmission. Values: 0dB, 2dB, 4dB, 6dB.</t>
+          <t>rach-power-ramping-step</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>rach-power-ramping-step</t>
+          <t>Power ramping step for preamble retransmission.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>RW</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>leaf</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>ENUMERATION</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>0dB, 2dB, 4dB, 6dB</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
+          <t>0dB 2dB 4dB 6dB</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>2dB</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>Random Access</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>FGR-RS0101</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
@@ -1169,71 +1261,81 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>bwp-inactivity-timer</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>Inactivity timer for returning to default BWP (ms). 0 disables the timer.</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>bwp-inactivity-timer</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>leaf</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>ms</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
         <is>
           <t>0..2560</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>2560</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>Bandwidth Part</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>FGR-BW0301</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
@@ -1247,71 +1349,81 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>bwp-initial-dl-bandwidth</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>Initial downlink BWP bandwidth in resource blocks.</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>bwp-initial-dl-bandwidth</t>
-        </is>
-      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>leaf</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>RB</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
         <is>
           <t>1..275</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>52</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>Bandwidth Part</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>FGR-BW0301</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
@@ -1325,67 +1437,77 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Time-to-trigger for event evaluation. Values: 0ms 40ms 64ms 80ms 100ms 128ms 160ms 256ms 320ms 480ms 512ms 640ms.</t>
+          <t>meas-time-to-trigger</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>meas-time-to-trigger</t>
+          <t>Time-to-trigger for event evaluation.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>RW</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>leaf</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>ENUMERATION</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>0ms 40ms 64ms 80ms 100ms 128ms 160ms 256ms 320ms 480ms 512ms 640ms</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
         <is>
           <t>100ms</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
         <is>
           <t>Cell</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>Handover</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>FGR-HO0102</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>

</xml_diff>